<commit_message>
updated tracker and gantt and hub to reflect new files
404 now fixed
</commit_message>
<xml_diff>
--- a/files/Spinney_Budget_Tracker_v5.xlsx
+++ b/files/Spinney_Budget_Tracker_v5.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="383">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -143,7 +143,7 @@
     <t xml:space="preserve">Snapshot</t>
   </si>
   <si>
-    <t xml:space="preserve">Week 8 — overall, still on plan, with one genuine new addition: a separate roofline works estimate (£2,100, after reclassifying its £40 rubbish line into the pooled fund) has surfaced, own scope and own budget, pushing PROJECT TOTAL to £69,428.99. Chimney and coping remain fully complete and settled (Gate 1 cleared 18 Aug). Decking is the active workstream: substructure under way on both sides plus the new shed area, the chimney pipe scare resolved with no cost, and labour payments tracking to quote once the cash discount is correctly applied. Materials pool is back under cap. Contingency now has four genuine draws (plus two more pending) but is still comfortably under its £5,000 cap. Nothing here suggests a budget problem.</t>
+    <t xml:space="preserve">Week 9 — overall, still on plan. Roofline works (£2,100) is a genuine new addition, own scope and own budget. Chimney and coping remain fully complete and settled (Gate 1 cleared 18 Aug). Decking is the active workstream: substructure re-planned to ~22 Sep across both sides plus the new shed area, board-laying to follow once Gates 2 and 3 clear. Materials pool is back under cap. Contingency has six genuine draws but is still comfortably under half-drawn. Nothing here suggests a budget problem.</t>
   </si>
   <si>
     <t xml:space="preserve">• Chimney</t>
@@ -194,6 +194,9 @@
     <t xml:space="preserve">£480.98 drawn of the £5,000 pot (condensation-prep £276.42 + chimney cowl upgrade £62.90 + V4 screw top-up £141.66) — £4,519.02 remaining. All three are genuine scope additions beyond the original quotes, which is exactly what this pot is for.</t>
   </si>
   <si>
+    <t xml:space="preserve">£622.64 drawn of the £5,000 pot (condensation-prep £276.42 + chimney cowl upgrade £62.90 + two V4 screw top-ups £283.32) — £4,377.36 remaining. All genuine scope additions beyond the original quotes, which is exactly what this pot is for.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Budget vs Actual — detail</t>
   </si>
   <si>
@@ -257,7 +260,7 @@
     <t xml:space="preserve">New scope, own budget — gutters, fascia/soffit, slates, barge boards. £40 rubbish removal reclassified to the pooled Rubbish removal fund. Not yet started or invoiced; quote used as placeholder actual until real costs land.</t>
   </si>
   <si>
-    <t xml:space="preserve">£480.98 drawn (condensation-prep £276.42 + chimney cowl £62.90 + V4 screw top-up £141.66) — £4,519.02 remaining. Variance here just means 'not yet drawn', not a saving.</t>
+    <t xml:space="preserve">£622.64 drawn of the £5,000 pot (condensation-prep £276.42 + chimney cowl £62.90 + V4 screw top-ups £283.32) — £4,377.36 remaining. Variance here just means 'not yet drawn', not a saving.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL (as spent/committed to date)</t>
@@ -698,21 +701,21 @@
     <t xml:space="preserve">Named purpose #9 — V4 screw top-up #2: 15 more boxes of Timberfix structural subframe screws (FH90P050), separate order from purpose #8</t>
   </si>
   <si>
+    <t xml:space="preserve">Paid, delivery scheduled 11 Sep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAID 10 Sep — invoice received. £141.66 used (matching purpose #8's confirmed rate: 15 x £7.87 + 20% VAT) — no invoice number/exact figure given this time, so this is inferred from the established pattern rather than confirmed from a document. Flag if the actual invoice differs. Delivery scheduled 11 Sep.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plant hire company (TBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Named purpose #10 — digger + barrow loader hire, one week (on hire until Thu 10 Sep). Mixed purpose: excavation for decking widening, side (a), AND new shed area, perpendicular to side (a)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Estimate</t>
   </si>
   <si>
-    <t xml:space="preserve">Ordered, not yet invoiced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordered 5 Sep (confirmed 6 Sep) — 15 boxes at £7.87/box, same unit price as purpose #8. Estimated £141.66 inc VAT (matching purpose #8's actual invoice pattern: 15 x £7.87 = £118.05 net + 20% VAT). Not yet paid — actual invoice will confirm. Pipe investigation (previously earmarked #9) resolved 4 Sep with no draw needed, freeing this slot.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plant hire company (TBC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Named purpose #10 — digger + barrow loader hire, one week (on hire until Thu 10 Sep). Mixed purpose: excavation for decking widening, side (a), AND new shed area, perpendicular to side (a)</t>
-  </si>
-  <si>
     <t xml:space="preserve">On hire, not yet invoiced</t>
   </si>
   <si>
@@ -1022,6 +1025,15 @@
     <t xml:space="preserve">Retires £2,222.22 of quoted value at the 10% cash discount (£2,000 paid = 90%). Not a full 25% stage — partial/interim payment. Total paid to date: £6,400 (Stage 1 £4,400 invoiced + this £2,000 cash). Quoted value remaining: £10,977.78.</t>
   </si>
   <si>
+    <t xml:space="preserve">TBC (no invoice number given)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V4 screw top-up #2 — 15 boxes structural subframe screws (named purpose #9)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice received and paid 10 Sep, delivery scheduled 11 Sep. Amount inferred from purpose #8's confirmed rate — no invoice number/exact figure given; flag if actual differs.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Skip Hire Log — pooled rubbish-removal drawdown</t>
   </si>
   <si>
@@ -1133,7 +1145,7 @@
     <t xml:space="preserve">Contingency Drawdown — £5,000 pot (agreed Lara/Luke, 1 Jul 2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Named purposes: fence move/repair labour · ~~soakaway fix before decking~~ CANCELLED 1 Sep, cost-benefit not worth it, nothing drawn · drainage by the garage · additional curved-decking labour · cement &amp; bricks · coping condensation-prep (£276.42, purpose #6) · chimney cowl upgrade (£62.90, purpose #7) · V4 screw top-up (£141.66, purpose #8) · V4 screw top-up #2 (est. £141.66, purpose #9, ordered 5 Sep, not yet invoiced) · digger + barrow loader hire (est. £530, purpose #10, on hire until 10 Sep, mixed purpose — side (a) decking widening + new shed excavation). Luke's labour from this pot invoiced at 10% discount (extended 20 Jul) — condensation-prep, the cowl, and both screw top-ups were/are bank transfer/direct paid, not cash, so no discount applies to any of them. Curved-decking extra labour discount status TBC. Pipe investigation (task 2.2) RESOLVED 4 Sep: no leaking pipe found.</t>
+    <t xml:space="preserve">Named purposes: fence move/repair labour · ~~soakaway fix before decking~~ CANCELLED 1 Sep, cost-benefit not worth it, nothing drawn · drainage by the garage · additional curved-decking labour · cement &amp; bricks · coping condensation-prep (£276.42, purpose #6) · chimney cowl upgrade (£62.90, purpose #7) · V4 screw top-up (£141.66, purpose #8) · V4 screw top-up #2 (£141.66, purpose #9, PAID 10 Sep, delivery 11 Sep) · digger + barrow loader hire (est. £530, purpose #10, on hire until 10 Sep, mixed purpose — side (a) decking widening + new shed excavation). Luke's labour from this pot invoiced at 10% discount (extended 20 Jul) — condensation-prep, the cowl, and both screw top-ups were/are bank transfer/direct paid, not cash, so no discount applies to any of them. Curved-decking extra labour discount status TBC. Pipe investigation (task 2.2) RESOLVED 4 Sep: no leaking pipe found.</t>
   </si>
   <si>
     <t xml:space="preserve">Opening pot:</t>
@@ -1161,13 +1173,16 @@
   </si>
   <si>
     <t xml:space="preserve">V4 Wood Flooring Ltd (V4FQ-17702)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V4 screw top-up #2 (named purpose #9) — PAID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd\ mmm\ yyyy"/>
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
@@ -1175,6 +1190,7 @@
     <numFmt numFmtId="168" formatCode="\£#,##0.00;&quot;-£&quot;#,##0.00"/>
     <numFmt numFmtId="169" formatCode="\£#,##0.00;[RED]&quot;-£&quot;#,##0.00"/>
     <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
   <fonts count="17">
     <font>
@@ -1418,7 +1434,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1696,6 +1712,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2084,15 +2104,15 @@
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A7,'Invoice Register'!$F:$F)</f>
-        <v>480.98</v>
+        <v>622.64</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A7,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>480.98</v>
+        <v>622.64</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">C7-D7</f>
-        <v>4519.02</v>
+        <v>4377.36</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>18</v>
@@ -2239,15 +2259,15 @@
       </c>
       <c r="D13" s="15" t="n">
         <f aca="false">D5+D6+D7</f>
-        <v>39109.97</v>
+        <v>39251.63</v>
       </c>
       <c r="E13" s="15" t="n">
         <f aca="false">E5+E6+E7</f>
-        <v>39109.97</v>
+        <v>39251.63</v>
       </c>
       <c r="F13" s="15" t="n">
         <f aca="false">F5+F6+F7</f>
-        <v>15719.02</v>
+        <v>15577.36</v>
       </c>
       <c r="G13" s="22"/>
     </row>
@@ -2285,15 +2305,15 @@
       </c>
       <c r="D15" s="28" t="n">
         <f aca="false">D11+D12+D13</f>
-        <v>39889.97</v>
+        <v>40031.63</v>
       </c>
       <c r="E15" s="28" t="n">
         <f aca="false">E11+E12+E13</f>
-        <v>39889.97</v>
+        <v>40031.63</v>
       </c>
       <c r="F15" s="28" t="n">
         <f aca="false">F11+F12+F13</f>
-        <v>18399.02</v>
+        <v>18257.36</v>
       </c>
       <c r="G15" s="27"/>
     </row>
@@ -2303,7 +2323,7 @@
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">'Contingency Drawdown'!$D$4</f>
-        <v>4519.02</v>
+        <v>4377.36</v>
       </c>
     </row>
   </sheetData>
@@ -2439,10 +2459,14 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2450,21 +2474,21 @@
         <v>3</v>
       </c>
       <c r="B17" s="35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D17" s="35" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E17" s="34" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B18" s="36" t="n">
         <v>3200</v>
@@ -2476,12 +2500,12 @@
         <v>0</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="38" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B19" s="39" t="n">
         <v>3800</v>
@@ -2493,12 +2517,12 @@
         <v>-190</v>
       </c>
       <c r="E19" s="38" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B20" s="36" t="n">
         <v>17600</v>
@@ -2510,12 +2534,12 @@
         <v>-11200</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B21" s="36" t="n">
         <v>32228.99</v>
@@ -2527,12 +2551,12 @@
         <v>0</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22" s="36" t="n">
         <v>3200</v>
@@ -2544,12 +2568,12 @@
         <v>0</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="38" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B23" s="39" t="n">
         <v>1130</v>
@@ -2561,12 +2585,12 @@
         <v>-9.31</v>
       </c>
       <c r="E23" s="38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B24" s="42" t="n">
         <v>1360</v>
@@ -2578,12 +2602,12 @@
         <v>-580</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B25" s="36" t="n">
         <v>2100</v>
@@ -2595,7 +2619,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2606,27 +2630,27 @@
         <v>5000</v>
       </c>
       <c r="C26" s="36" t="n">
-        <v>480.98</v>
+        <v>622.64</v>
       </c>
       <c r="D26" s="41" t="n">
-        <v>-4519.02</v>
+        <v>-4377.36</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>69618.99</v>
       </c>
       <c r="C27" s="1" t="n">
-        <v>53120.66</v>
+        <v>53262.32</v>
       </c>
       <c r="D27" s="45" t="n">
-        <v>-16498.33</v>
+        <v>-16356.67</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2638,18 +2662,18 @@
     </row>
     <row r="29" customFormat="false" ht="149.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="47" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="33" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C32" s="48" t="n">
         <v>4700</v>
@@ -2657,7 +2681,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C33" s="48" t="n">
         <v>5310</v>
@@ -2665,7 +2689,7 @@
     </row>
     <row r="34" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C34" s="48" t="n">
         <v>17600</v>
@@ -2673,7 +2697,7 @@
     </row>
     <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="33" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C35" s="48" t="n">
         <v>32228.99</v>
@@ -2681,7 +2705,7 @@
     </row>
     <row r="36" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C36" s="48" t="n">
         <v>1130</v>
@@ -2689,7 +2713,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="33" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C37" s="48" t="n">
         <v>1360</v>
@@ -2697,7 +2721,7 @@
     </row>
     <row r="38" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="33" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C38" s="48" t="n">
         <v>5000</v>
@@ -2705,7 +2729,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C39" s="48" t="n">
         <v>2100</v>
@@ -2713,7 +2737,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="50" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B40" s="51"/>
       <c r="C40" s="52" t="n">
@@ -2725,7 +2749,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="50" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B41" s="51"/>
       <c r="C41" s="52" t="n">
@@ -2737,7 +2761,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="50" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B42" s="51"/>
       <c r="C42" s="53" t="n">
@@ -2788,35 +2812,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>9</v>
@@ -2830,19 +2854,19 @@
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F5" s="18" t="n">
         <v>32228.99</v>
       </c>
       <c r="G5" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H5" s="8"/>
     </row>
@@ -2851,25 +2875,25 @@
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>2000</v>
       </c>
       <c r="G6" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2877,25 +2901,25 @@
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>1200</v>
       </c>
       <c r="G7" s="56" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2906,22 +2930,22 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>3200</v>
       </c>
       <c r="G8" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2932,22 +2956,22 @@
         <v>21</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>1710</v>
       </c>
       <c r="G9" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2958,22 +2982,22 @@
         <v>21</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>1900</v>
       </c>
       <c r="G10" s="56" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2984,22 +3008,22 @@
         <v>16</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="57" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3010,22 +3034,22 @@
         <v>13</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>17600</v>
       </c>
       <c r="G12" s="56" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3036,22 +3060,22 @@
         <v>23</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>1130</v>
       </c>
       <c r="G13" s="56" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,22 +3086,22 @@
         <v>16</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>5000</v>
       </c>
       <c r="G14" s="56" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3088,22 +3112,22 @@
         <v>16</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="55" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3114,22 +3138,22 @@
         <v>26</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>27</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F16" s="19" t="n">
         <v>1360</v>
       </c>
       <c r="G16" s="56" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3140,22 +3164,22 @@
         <v>29</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D17" s="54" t="s">
         <v>14</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F17" s="19" t="n">
         <v>2100</v>
       </c>
       <c r="G17" s="54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3164,7 +3188,7 @@
       <c r="C18" s="54"/>
       <c r="D18" s="54"/>
       <c r="E18" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F18" s="58" t="n">
         <f aca="false">SUM(F5:F17)</f>
@@ -3179,7 +3203,7 @@
       <c r="C19" s="59"/>
       <c r="D19" s="59"/>
       <c r="E19" s="60" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F19" s="61" t="n">
         <f aca="false">Summary!$C$15</f>
@@ -3194,7 +3218,7 @@
       <c r="C20" s="59"/>
       <c r="D20" s="59"/>
       <c r="E20" s="60" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F20" s="61" t="n">
         <f aca="false">F18-F19</f>
@@ -3246,12 +3270,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3262,22 +3286,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -3288,10 +3312,10 @@
         <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D5" s="58"/>
       <c r="E5" s="58"/>
@@ -3299,13 +3323,13 @@
         <v>3200</v>
       </c>
       <c r="G5" s="58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3313,10 +3337,10 @@
         <v>19</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D6" s="58"/>
       <c r="E6" s="58"/>
@@ -3324,13 +3348,13 @@
         <v>1500</v>
       </c>
       <c r="G6" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3341,7 +3365,7 @@
         <v>24</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D7" s="58"/>
       <c r="E7" s="58"/>
@@ -3349,10 +3373,10 @@
         <v>480</v>
       </c>
       <c r="G7" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I7" s="11"/>
     </row>
@@ -3361,10 +3385,10 @@
         <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D8" s="58"/>
       <c r="E8" s="58"/>
@@ -3372,13 +3396,13 @@
         <v>0</v>
       </c>
       <c r="G8" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3386,10 +3410,10 @@
         <v>21</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D9" s="58"/>
       <c r="E9" s="58"/>
@@ -3397,13 +3421,13 @@
         <v>3610</v>
       </c>
       <c r="G9" s="58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3411,10 +3435,10 @@
         <v>21</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D10" s="58"/>
       <c r="E10" s="58"/>
@@ -3422,13 +3446,13 @@
         <v>1700</v>
       </c>
       <c r="G10" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3439,7 +3463,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D11" s="58"/>
       <c r="E11" s="58"/>
@@ -3447,10 +3471,10 @@
         <v>650</v>
       </c>
       <c r="G11" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I11" s="11"/>
     </row>
@@ -3459,10 +3483,10 @@
         <v>21</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D12" s="58"/>
       <c r="E12" s="58"/>
@@ -3470,13 +3494,13 @@
         <v>0</v>
       </c>
       <c r="G12" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3484,10 +3508,10 @@
         <v>13</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D13" s="58"/>
       <c r="E13" s="58"/>
@@ -3495,13 +3519,13 @@
         <v>17600</v>
       </c>
       <c r="G13" s="58" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3509,10 +3533,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D14" s="58"/>
       <c r="E14" s="58"/>
@@ -3520,13 +3544,13 @@
         <v>0</v>
       </c>
       <c r="G14" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3534,10 +3558,10 @@
         <v>10</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D15" s="58" t="n">
         <v>230</v>
@@ -3549,10 +3573,10 @@
         <v>15292.7</v>
       </c>
       <c r="G15" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I15" s="11"/>
     </row>
@@ -3561,10 +3585,10 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D16" s="58" t="n">
         <v>18</v>
@@ -3576,10 +3600,10 @@
         <v>1045.62</v>
       </c>
       <c r="G16" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -3588,10 +3612,10 @@
         <v>10</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D17" s="58" t="n">
         <v>15</v>
@@ -3603,13 +3627,13 @@
         <v>1083.75</v>
       </c>
       <c r="G17" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3617,10 +3641,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D18" s="58" t="n">
         <v>15</v>
@@ -3632,10 +3656,10 @@
         <v>898.35</v>
       </c>
       <c r="G18" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I18" s="11"/>
     </row>
@@ -3644,10 +3668,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D19" s="58" t="n">
         <v>24</v>
@@ -3659,10 +3683,10 @@
         <v>770</v>
       </c>
       <c r="G19" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I19" s="11"/>
     </row>
@@ -3671,10 +3695,10 @@
         <v>10</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D20" s="58" t="n">
         <v>6</v>
@@ -3686,10 +3710,10 @@
         <v>61.5</v>
       </c>
       <c r="G20" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I20" s="11"/>
     </row>
@@ -3698,10 +3722,10 @@
         <v>10</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D21" s="58" t="n">
         <v>266</v>
@@ -3713,13 +3737,13 @@
         <v>7554.4</v>
       </c>
       <c r="G21" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3727,10 +3751,10 @@
         <v>10</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D22" s="58" t="n">
         <v>16</v>
@@ -3742,13 +3766,13 @@
         <v>125.92</v>
       </c>
       <c r="G22" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I22" s="11" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3756,10 +3780,10 @@
         <v>10</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D23" s="58" t="n">
         <v>1</v>
@@ -3771,10 +3795,10 @@
         <v>15</v>
       </c>
       <c r="G23" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I23" s="11"/>
     </row>
@@ -3783,10 +3807,10 @@
         <v>10</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D24" s="58" t="n">
         <v>1</v>
@@ -3798,10 +3822,10 @@
         <v>10.25</v>
       </c>
       <c r="G24" s="58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I24" s="11"/>
     </row>
@@ -3810,10 +3834,10 @@
         <v>10</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D25" s="58"/>
       <c r="E25" s="58"/>
@@ -3821,13 +3845,13 @@
         <v>5371.5</v>
       </c>
       <c r="G25" s="58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3835,10 +3859,10 @@
         <v>16</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D26" s="58"/>
       <c r="E26" s="58"/>
@@ -3849,10 +3873,10 @@
         <v>17</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3863,7 +3887,7 @@
         <v>14</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D27" s="58"/>
       <c r="E27" s="58"/>
@@ -3871,13 +3895,13 @@
         <v>250</v>
       </c>
       <c r="G27" s="58" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3885,10 +3909,10 @@
         <v>16</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D28" s="58" t="n">
         <v>1</v>
@@ -3900,13 +3924,13 @@
         <v>62.9</v>
       </c>
       <c r="G28" s="58" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3914,10 +3938,10 @@
         <v>23</v>
       </c>
       <c r="B29" s="54" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D29" s="54"/>
       <c r="E29" s="54"/>
@@ -3925,20 +3949,20 @@
         <v>481.26</v>
       </c>
       <c r="G29" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H29" s="54" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="54"/>
       <c r="B30" s="54"/>
       <c r="C30" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D30" s="54"/>
       <c r="E30" s="54"/>
@@ -3946,13 +3970,13 @@
         <v>0</v>
       </c>
       <c r="G30" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H30" s="54" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3963,7 +3987,7 @@
         <v>11</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D31" s="54"/>
       <c r="E31" s="54"/>
@@ -3971,13 +3995,13 @@
         <v>141.66</v>
       </c>
       <c r="G31" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H31" s="54" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3988,7 +4012,7 @@
         <v>11</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D32" s="54"/>
       <c r="E32" s="54"/>
@@ -3996,7 +4020,7 @@
         <v>141.66</v>
       </c>
       <c r="G32" s="54" t="s">
-        <v>223</v>
+        <v>102</v>
       </c>
       <c r="H32" s="54" t="s">
         <v>224</v>
@@ -4021,13 +4045,13 @@
         <v>530</v>
       </c>
       <c r="G33" s="54" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="H33" s="54" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4035,10 +4059,10 @@
         <v>26</v>
       </c>
       <c r="B34" s="54" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D34" s="54"/>
       <c r="E34" s="54"/>
@@ -4046,13 +4070,13 @@
         <v>350</v>
       </c>
       <c r="G34" s="54" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H34" s="54" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I34" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4063,7 +4087,7 @@
         <v>14</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D35" s="54"/>
       <c r="E35" s="54"/>
@@ -4071,13 +4095,13 @@
         <v>1600</v>
       </c>
       <c r="G35" s="54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H35" s="54" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I35" s="20" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4088,7 +4112,7 @@
         <v>14</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D36" s="54"/>
       <c r="E36" s="54"/>
@@ -4096,13 +4120,13 @@
         <v>150</v>
       </c>
       <c r="G36" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H36" s="54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I36" s="20" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4113,7 +4137,7 @@
         <v>14</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D37" s="54"/>
       <c r="E37" s="54"/>
@@ -4121,13 +4145,13 @@
         <v>350</v>
       </c>
       <c r="G37" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H37" s="54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I37" s="20" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4138,7 +4162,7 @@
         <v>14</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D38" s="54"/>
       <c r="E38" s="54"/>
@@ -4146,18 +4170,18 @@
         <v>40</v>
       </c>
       <c r="G38" s="54" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H38" s="54" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I38" s="20" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C39" s="63" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F39" s="64" t="n">
         <f aca="false">SUM(F5:F38)</f>
@@ -4180,7 +4204,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
@@ -4194,17 +4218,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -4213,19 +4237,19 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -4242,10 +4266,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F5" s="18" t="n">
         <v>32228.99</v>
@@ -4254,10 +4278,10 @@
         <v>46212</v>
       </c>
       <c r="H5" s="54" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4268,13 +4292,13 @@
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>311.98</v>
@@ -4283,10 +4307,10 @@
         <v>46223</v>
       </c>
       <c r="H6" s="54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4297,13 +4321,13 @@
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>111.71</v>
@@ -4312,10 +4336,10 @@
         <v>46223</v>
       </c>
       <c r="H7" s="54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4326,13 +4350,13 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>937.5</v>
@@ -4341,10 +4365,10 @@
         <v>46223</v>
       </c>
       <c r="H8" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4358,10 +4382,10 @@
         <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>3088.3</v>
@@ -4370,10 +4394,10 @@
         <v>46227</v>
       </c>
       <c r="H9" s="54" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4384,13 +4408,13 @@
         <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>162.96</v>
@@ -4399,10 +4423,10 @@
         <v>46225</v>
       </c>
       <c r="H10" s="54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4413,13 +4437,13 @@
         <v>23</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>148.53</v>
@@ -4428,10 +4452,10 @@
         <v>46238</v>
       </c>
       <c r="H11" s="54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4445,10 +4469,10 @@
         <v>14</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>1710</v>
@@ -4457,10 +4481,10 @@
         <v>46241</v>
       </c>
       <c r="H12" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4471,13 +4495,13 @@
         <v>16</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>62.9</v>
@@ -4486,10 +4510,10 @@
         <v>46244</v>
       </c>
       <c r="H13" s="54" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4500,13 +4524,13 @@
         <v>26</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>344.16</v>
@@ -4515,10 +4539,10 @@
         <v>46244</v>
       </c>
       <c r="H14" s="54" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4529,13 +4553,13 @@
         <v>26</v>
       </c>
       <c r="C15" s="67" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D15" s="67" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E15" s="68" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F15" s="69" t="n">
         <v>-344.16</v>
@@ -4547,7 +4571,7 @@
         <v>17</v>
       </c>
       <c r="I15" s="68" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4558,13 +4582,13 @@
         <v>26</v>
       </c>
       <c r="C16" s="67" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D16" s="67" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E16" s="68" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F16" s="69" t="n">
         <v>390</v>
@@ -4573,10 +4597,10 @@
         <v>46246</v>
       </c>
       <c r="H16" s="67" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I16" s="68" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4587,13 +4611,13 @@
         <v>26</v>
       </c>
       <c r="C17" s="67" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D17" s="67" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E17" s="68" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F17" s="69" t="n">
         <v>390</v>
@@ -4602,10 +4626,10 @@
         <v>46246</v>
       </c>
       <c r="H17" s="67" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I17" s="68" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4619,10 +4643,10 @@
         <v>14</v>
       </c>
       <c r="D18" s="67" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E18" s="68" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F18" s="69" t="n">
         <v>1900</v>
@@ -4631,10 +4655,10 @@
         <v>46248</v>
       </c>
       <c r="H18" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I18" s="68" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4648,10 +4672,10 @@
         <v>14</v>
       </c>
       <c r="D19" s="67" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E19" s="68" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F19" s="69" t="n">
         <v>250</v>
@@ -4660,10 +4684,10 @@
         <v>46248</v>
       </c>
       <c r="H19" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I19" s="68" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4674,13 +4698,13 @@
         <v>23</v>
       </c>
       <c r="C20" s="67" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D20" s="67" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E20" s="68" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F20" s="69" t="n">
         <v>47.99</v>
@@ -4689,10 +4713,10 @@
         <v>46250</v>
       </c>
       <c r="H20" s="67" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="I20" s="68" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4703,13 +4727,13 @@
         <v>23</v>
       </c>
       <c r="C21" s="67" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D21" s="67" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E21" s="68" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F21" s="69" t="n">
         <v>481.28</v>
@@ -4718,10 +4742,10 @@
         <v>46252</v>
       </c>
       <c r="H21" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I21" s="68" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4732,13 +4756,13 @@
         <v>23</v>
       </c>
       <c r="C22" s="67" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D22" s="67" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E22" s="68" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F22" s="69" t="n">
         <v>-72.23</v>
@@ -4747,10 +4771,10 @@
         <v>46253</v>
       </c>
       <c r="H22" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I22" s="68" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4761,13 +4785,13 @@
         <v>16</v>
       </c>
       <c r="C23" s="67" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D23" s="67" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E23" s="68" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F23" s="69" t="n">
         <v>26.42</v>
@@ -4776,10 +4800,10 @@
         <v>46252</v>
       </c>
       <c r="H23" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I23" s="68" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4790,13 +4814,13 @@
         <v>23</v>
       </c>
       <c r="C24" s="67" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D24" s="67" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E24" s="68" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F24" s="69" t="n">
         <v>40.18</v>
@@ -4805,10 +4829,10 @@
         <v>46252</v>
       </c>
       <c r="H24" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I24" s="68" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4822,10 +4846,10 @@
         <v>14</v>
       </c>
       <c r="D25" s="67" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E25" s="68" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F25" s="69" t="n">
         <v>4400</v>
@@ -4834,10 +4858,10 @@
         <v>46254</v>
       </c>
       <c r="H25" s="67" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I25" s="68" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4848,13 +4872,13 @@
         <v>21</v>
       </c>
       <c r="C26" s="54" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D26" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F26" s="54" t="n">
         <v>1062.5</v>
@@ -4863,10 +4887,10 @@
         <v>46223</v>
       </c>
       <c r="H26" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4877,13 +4901,13 @@
         <v>19</v>
       </c>
       <c r="C27" s="54" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D27" s="54" t="s">
         <v>17</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F27" s="54" t="n">
         <v>562.5</v>
@@ -4892,10 +4916,10 @@
         <v>46252</v>
       </c>
       <c r="H27" s="54" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4906,13 +4930,13 @@
         <v>21</v>
       </c>
       <c r="C28" s="54" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D28" s="54" t="s">
         <v>17</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F28" s="54" t="n">
         <v>637.5</v>
@@ -4921,10 +4945,10 @@
         <v>46252</v>
       </c>
       <c r="H28" s="54" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4938,10 +4962,10 @@
         <v>11</v>
       </c>
       <c r="D29" s="54" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F29" s="54" t="n">
         <v>141.66</v>
@@ -4950,10 +4974,10 @@
         <v>46258</v>
       </c>
       <c r="H29" s="54" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="108.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4967,10 +4991,10 @@
         <v>14</v>
       </c>
       <c r="D30" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F30" s="54" t="n">
         <v>2000</v>
@@ -4979,10 +5003,39 @@
         <v>46269</v>
       </c>
       <c r="H30" s="54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>330</v>
+        <v>331</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="70" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B31" s="54" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="54" t="s">
+        <v>332</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="F31" s="54" t="n">
+        <v>141.66</v>
+      </c>
+      <c r="G31" s="70" t="n">
+        <v>46275</v>
+      </c>
+      <c r="H31" s="54" t="s">
+        <v>203</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -5014,47 +5067,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="B4" s="70" t="n">
+        <v>337</v>
+      </c>
+      <c r="B4" s="71" t="n">
         <v>1360</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="D4" s="71" t="n">
+        <v>338</v>
+      </c>
+      <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
         <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5062,13 +5115,13 @@
         <v>46244</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>344.16</v>
@@ -5083,13 +5136,13 @@
         <v>46245</v>
       </c>
       <c r="B9" s="68" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C9" s="68" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="D9" s="68" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="E9" s="69" t="n">
         <v>-344.16</v>
@@ -5104,13 +5157,13 @@
         <v>46245</v>
       </c>
       <c r="B10" s="68" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D10" s="68" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E10" s="69" t="n">
         <v>390</v>
@@ -5125,13 +5178,13 @@
         <v>46246</v>
       </c>
       <c r="B11" s="68" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C11" s="68" t="s">
+        <v>350</v>
+      </c>
+      <c r="D11" s="68" t="s">
         <v>346</v>
-      </c>
-      <c r="D11" s="68" t="s">
-        <v>342</v>
       </c>
       <c r="E11" s="69" t="n">
         <v>390</v>
@@ -5146,13 +5199,13 @@
         <v>46273</v>
       </c>
       <c r="B12" s="68" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="C12" s="68" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D12" s="67" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="E12" s="69" t="n">
         <v>350</v>
@@ -5170,7 +5223,7 @@
         <v>14</v>
       </c>
       <c r="C13" s="68" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="D13" s="67" t="s">
         <v>29</v>
@@ -5184,132 +5237,132 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="72"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="73"/>
-      <c r="E14" s="74"/>
+      <c r="A14" s="73"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="74"/>
+      <c r="E14" s="75"/>
       <c r="F14" s="10" t="str">
         <f aca="false">IF(E14="","",$B$4-SUM($E$8:E14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="72"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="74"/>
+      <c r="A15" s="73"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74"/>
+      <c r="E15" s="75"/>
       <c r="F15" s="10" t="str">
         <f aca="false">IF(E15="","",$B$4-SUM($E$8:E15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="72"/>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="73"/>
-      <c r="E16" s="74"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="75"/>
       <c r="F16" s="10" t="str">
         <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="72"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="73"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="74"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="75"/>
       <c r="F17" s="10" t="str">
         <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="72"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="74"/>
+      <c r="A18" s="73"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="75"/>
       <c r="F18" s="10" t="str">
         <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="72"/>
-      <c r="B19" s="73"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="73"/>
-      <c r="E19" s="74"/>
+      <c r="A19" s="73"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="75"/>
       <c r="F19" s="10" t="str">
         <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="72"/>
-      <c r="B20" s="73"/>
-      <c r="C20" s="73"/>
-      <c r="D20" s="73"/>
-      <c r="E20" s="74"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="75"/>
       <c r="F20" s="10" t="str">
         <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="72"/>
-      <c r="B21" s="73"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="73"/>
-      <c r="E21" s="74"/>
+      <c r="A21" s="73"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="74"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="75"/>
       <c r="F21" s="10" t="str">
         <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="72"/>
-      <c r="B22" s="73"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="73"/>
-      <c r="E22" s="74"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="74"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="75"/>
       <c r="F22" s="10" t="str">
         <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="72"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="74"/>
+      <c r="A23" s="73"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="75"/>
       <c r="F23" s="10" t="str">
         <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="72"/>
-      <c r="B24" s="73"/>
-      <c r="C24" s="73"/>
-      <c r="D24" s="73"/>
-      <c r="E24" s="74"/>
+      <c r="A24" s="73"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="75"/>
       <c r="F24" s="10" t="str">
         <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="72"/>
-      <c r="B25" s="73"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="74"/>
+      <c r="A25" s="73"/>
+      <c r="B25" s="74"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="75"/>
       <c r="F25" s="10" t="str">
         <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
         <v/>
@@ -5344,47 +5397,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="B4" s="70" t="n">
+        <v>337</v>
+      </c>
+      <c r="B4" s="71" t="n">
         <v>1130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="D4" s="71" t="n">
+        <v>338</v>
+      </c>
+      <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
         <v>-62.9000000000001</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5392,13 +5445,13 @@
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="E8" s="18" t="n">
         <v>311.98</v>
@@ -5413,13 +5466,13 @@
         <v>46225</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="E9" s="18" t="n">
         <v>162.96</v>
@@ -5434,13 +5487,13 @@
         <v>46238</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="D10" s="54" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="E10" s="18" t="n">
         <v>148.53</v>
@@ -5455,13 +5508,13 @@
         <v>46250</v>
       </c>
       <c r="B11" s="67" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D11" s="68" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E11" s="69" t="n">
         <v>47.99</v>
@@ -5476,13 +5529,13 @@
         <v>46251</v>
       </c>
       <c r="B12" s="68" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C12" s="68" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="D12" s="67" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="E12" s="69" t="n">
         <v>481.26</v>
@@ -5508,13 +5561,13 @@
         <v>46244</v>
       </c>
       <c r="B14" s="68" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="C14" s="68" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="D14" s="67" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="E14" s="69" t="n">
         <v>40.18</v>
@@ -5536,110 +5589,110 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="72"/>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="73"/>
-      <c r="E16" s="74"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="74"/>
+      <c r="E16" s="75"/>
       <c r="F16" s="10" t="str">
         <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="72"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="73"/>
-      <c r="D17" s="73"/>
-      <c r="E17" s="74"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="75"/>
       <c r="F17" s="10" t="str">
         <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="72"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="73"/>
-      <c r="E18" s="74"/>
+      <c r="A18" s="73"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="74"/>
+      <c r="E18" s="75"/>
       <c r="F18" s="10" t="str">
         <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="72"/>
-      <c r="B19" s="73"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="73"/>
-      <c r="E19" s="74"/>
+      <c r="A19" s="73"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="74"/>
+      <c r="E19" s="75"/>
       <c r="F19" s="10" t="str">
         <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="72"/>
-      <c r="B20" s="73"/>
-      <c r="C20" s="73"/>
-      <c r="D20" s="73"/>
-      <c r="E20" s="74"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="74"/>
+      <c r="E20" s="75"/>
       <c r="F20" s="10" t="str">
         <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="72"/>
-      <c r="B21" s="73"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="73"/>
-      <c r="E21" s="74"/>
+      <c r="A21" s="73"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="74"/>
+      <c r="D21" s="74"/>
+      <c r="E21" s="75"/>
       <c r="F21" s="10" t="str">
         <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="72"/>
-      <c r="B22" s="73"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="73"/>
-      <c r="E22" s="74"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="74"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="74"/>
+      <c r="E22" s="75"/>
       <c r="F22" s="10" t="str">
         <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="72"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="74"/>
+      <c r="A23" s="73"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="75"/>
       <c r="F23" s="10" t="str">
         <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="72"/>
-      <c r="B24" s="73"/>
-      <c r="C24" s="73"/>
-      <c r="D24" s="73"/>
-      <c r="E24" s="74"/>
+      <c r="A24" s="73"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="75"/>
       <c r="F24" s="10" t="str">
         <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="72"/>
-      <c r="B25" s="73"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="73"/>
-      <c r="E25" s="74"/>
+      <c r="A25" s="73"/>
+      <c r="B25" s="74"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="75"/>
       <c r="F25" s="10" t="str">
         <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
         <v/>
@@ -5672,44 +5725,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="B4" s="70" t="n">
+        <v>373</v>
+      </c>
+      <c r="B4" s="71" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
-      </c>
-      <c r="D4" s="71" t="n">
+        <v>338</v>
+      </c>
+      <c r="D4" s="72" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
-        <v>4519.02</v>
+        <v>4377.36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5717,10 +5770,10 @@
         <v>46248</v>
       </c>
       <c r="B8" s="68" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C8" s="68" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="D8" s="69" t="n">
         <v>250</v>
@@ -5735,10 +5788,10 @@
         <v>46251</v>
       </c>
       <c r="B9" s="68" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="C9" s="68" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D9" s="69" t="n">
         <v>26.42</v>
@@ -5753,10 +5806,10 @@
         <v>46251</v>
       </c>
       <c r="B10" s="68" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="D10" s="69" t="n">
         <v>62.9</v>
@@ -5771,10 +5824,10 @@
         <v>46258</v>
       </c>
       <c r="B11" s="68" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="D11" s="69" t="n">
         <v>141.66</v>
@@ -5785,140 +5838,148 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="72"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="73"/>
-      <c r="D12" s="74"/>
-      <c r="E12" s="10" t="str">
+      <c r="A12" s="66" t="n">
+        <v>46275</v>
+      </c>
+      <c r="B12" s="68" t="s">
+        <v>382</v>
+      </c>
+      <c r="C12" s="68" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="69" t="n">
+        <v>141.66</v>
+      </c>
+      <c r="E12" s="10" t="n">
         <f aca="false">IF(D12="","",$B$4-SUM($D$8:D12))</f>
-        <v/>
+        <v>4377.36</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="72"/>
-      <c r="B13" s="73"/>
-      <c r="C13" s="73"/>
-      <c r="D13" s="74"/>
+      <c r="A13" s="73"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="75"/>
       <c r="E13" s="10" t="str">
         <f aca="false">IF(D13="","",$B$4-SUM($D$8:D13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="72"/>
-      <c r="B14" s="73"/>
-      <c r="C14" s="73"/>
-      <c r="D14" s="74"/>
+      <c r="A14" s="73"/>
+      <c r="B14" s="74"/>
+      <c r="C14" s="74"/>
+      <c r="D14" s="75"/>
       <c r="E14" s="10" t="str">
         <f aca="false">IF(D14="","",$B$4-SUM($D$8:D14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="72"/>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="74"/>
+      <c r="A15" s="73"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="D15" s="75"/>
       <c r="E15" s="10" t="str">
         <f aca="false">IF(D15="","",$B$4-SUM($D$8:D15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="72"/>
-      <c r="B16" s="73"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="74"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="74"/>
+      <c r="C16" s="74"/>
+      <c r="D16" s="75"/>
       <c r="E16" s="10" t="str">
         <f aca="false">IF(D16="","",$B$4-SUM($D$8:D16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="72"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="73"/>
-      <c r="D17" s="74"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="75"/>
       <c r="E17" s="10" t="str">
         <f aca="false">IF(D17="","",$B$4-SUM($D$8:D17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="72"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="73"/>
-      <c r="D18" s="74"/>
+      <c r="A18" s="73"/>
+      <c r="B18" s="74"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="75"/>
       <c r="E18" s="10" t="str">
         <f aca="false">IF(D18="","",$B$4-SUM($D$8:D18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="72"/>
-      <c r="B19" s="73"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="74"/>
+      <c r="A19" s="73"/>
+      <c r="B19" s="74"/>
+      <c r="C19" s="74"/>
+      <c r="D19" s="75"/>
       <c r="E19" s="10" t="str">
         <f aca="false">IF(D19="","",$B$4-SUM($D$8:D19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="72"/>
-      <c r="B20" s="73"/>
-      <c r="C20" s="73"/>
-      <c r="D20" s="74"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="74"/>
+      <c r="C20" s="74"/>
+      <c r="D20" s="75"/>
       <c r="E20" s="10" t="str">
         <f aca="false">IF(D20="","",$B$4-SUM($D$8:D20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="72"/>
-      <c r="B21" s="73"/>
-      <c r="C21" s="73"/>
-      <c r="D21" s="74"/>
+      <c r="A21" s="73"/>
+      <c r="B21" s="74"/>
+      <c r="C21" s="74"/>
+      <c r="D21" s="75"/>
       <c r="E21" s="10" t="str">
         <f aca="false">IF(D21="","",$B$4-SUM($D$8:D21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="72"/>
-      <c r="B22" s="73"/>
-      <c r="C22" s="73"/>
-      <c r="D22" s="74"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="74"/>
+      <c r="C22" s="74"/>
+      <c r="D22" s="75"/>
       <c r="E22" s="10" t="str">
         <f aca="false">IF(D22="","",$B$4-SUM($D$8:D22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="72"/>
-      <c r="B23" s="73"/>
-      <c r="C23" s="73"/>
-      <c r="D23" s="74"/>
+      <c r="A23" s="73"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="75"/>
       <c r="E23" s="10" t="str">
         <f aca="false">IF(D23="","",$B$4-SUM($D$8:D23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="72"/>
-      <c r="B24" s="73"/>
-      <c r="C24" s="73"/>
-      <c r="D24" s="74"/>
+      <c r="A24" s="73"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="75"/>
       <c r="E24" s="10" t="str">
         <f aca="false">IF(D24="","",$B$4-SUM($D$8:D24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="72"/>
-      <c r="B25" s="73"/>
-      <c r="C25" s="73"/>
-      <c r="D25" s="74"/>
+      <c r="A25" s="73"/>
+      <c r="B25" s="74"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="75"/>
       <c r="E25" s="10" t="str">
         <f aca="false">IF(D25="","",$B$4-SUM($D$8:D25))</f>
         <v/>

</xml_diff>